<commit_message>
Show rejected imports and add demo files
A file with errors shows that nothing was imported and lists the rows;
a successful import shows how many students were added. docs/demo has
a valid file and one with errors.
</commit_message>
<xml_diff>
--- a/docs/demo/telebeler.xlsx
+++ b/docs/demo/telebeler.xlsx
@@ -1,113 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Tələbələr" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
-  <si>
-    <t>first_name</t>
-  </si>
-  <si>
-    <t>last_name</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>Elvin</t>
-  </si>
-  <si>
-    <t>Məmmədli</t>
-  </si>
-  <si>
-    <t>elvin.memmedli.demo@abb.local</t>
-  </si>
-  <si>
-    <t>Nərmin</t>
-  </si>
-  <si>
-    <t>Hüseynova</t>
-  </si>
-  <si>
-    <t>nermin.huseynova.demo@abb.local</t>
-  </si>
-  <si>
-    <t>Kamran</t>
-  </si>
-  <si>
-    <t>Əlizadə</t>
-  </si>
-  <si>
-    <t>kamran.alizade.demo@abb.local</t>
-  </si>
-  <si>
-    <t>Səadət</t>
-  </si>
-  <si>
-    <t>Qasımova</t>
-  </si>
-  <si>
-    <t>seadet.qasimova.demo@abb.local</t>
-  </si>
-  <si>
-    <t>Orxan</t>
-  </si>
-  <si>
-    <t>Babayev</t>
-  </si>
-  <si>
-    <t>orxan.babayev.demo@abb.local</t>
-  </si>
-  <si>
-    <t>Ramil</t>
-  </si>
-  <si>
-    <t>Nəbiyev</t>
-  </si>
-  <si>
-    <t>ramil-email-yanlis</t>
-  </si>
-  <si>
-    <t>Rəşad</t>
-  </si>
-  <si>
-    <t>Hüseynov</t>
-  </si>
-  <si>
-    <t>rashad.huseynov@abb.local</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -126,13 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -211,7 +199,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -246,7 +233,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -422,118 +408,139 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="37.705" bestFit="true" customWidth="true" style="0"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>last_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Elvin</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Məmmədli</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>elvin.memmedli.demo@abb.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Nərmin</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Hüseynova</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>nermin.huseynova.demo@abb.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kamran</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Əlizadə</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>kamran.alizade.demo@abb.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Səadət</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Qasımova</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>seadet.qasimova.demo@abb.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Orxan</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Babayev</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>orxan.babayev.demo@abb.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ceyhun</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rzayev</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>student@abb.local</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>